<commit_message>
GiftLogs Sept 26 -24
</commit_message>
<xml_diff>
--- a/TestData/LV_T1525_ApproveGiftsDenySelectedToDenyTheGiftsFromPendingList.xlsx
+++ b/TestData/LV_T1525_ApproveGiftsDenySelectedToDenyTheGiftsFromPendingList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BACD183-A463-453B-944E-2A21E0F4EFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8FF45C3-AA39-4878-9EBC-BD83D0328C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
   <si>
     <t>Client Gift Pre-approval</t>
   </si>
@@ -72,9 +72,6 @@
     <t>ContactName</t>
   </si>
   <si>
-    <t>Test External</t>
-  </si>
-  <si>
     <t>CongratulationsMsg</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
     <t>StandardTestCompany</t>
   </si>
   <si>
-    <t>Julie Carthane</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -169,6 +163,9 @@
   </si>
   <si>
     <t>GroupName</t>
+  </si>
+  <si>
+    <t>Giftlog Contact</t>
   </si>
 </sst>
 </file>
@@ -516,18 +513,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -543,12 +540,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -566,17 +563,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -597,7 +594,7 @@
     <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
@@ -610,7 +607,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
@@ -619,7 +616,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
@@ -637,16 +634,16 @@
         <v>1</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -654,16 +651,16 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -672,25 +669,25 @@
         <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="J2" t="s">
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="N2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -716,39 +713,39 @@
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -766,12 +763,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -786,12 +783,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>